<commit_message>
Excel y Word Máquina 2
</commit_message>
<xml_diff>
--- a/Docs/ISIS1225 - Tablas de Datos Lab 4 - Maquina 2 Sarah González Almario.xlsx
+++ b/Docs/ISIS1225 - Tablas de Datos Lab 4 - Maquina 2 Sarah González Almario.xlsx
@@ -8713,7 +8713,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5B14742-4EBB-4241-AC8A-0E5F24F7BB7B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{D5B14742-4EBB-4241-AC8A-0E5F24F7BB7B}">
   <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
@@ -8770,12 +8770,24 @@
         <f>Table1[[#This Row],[Porcentaje de la muestra '[pct']]]*10000</f>
         <v>50</v>
       </c>
-      <c r="C3" s="4"/>
-      <c r="D3" s="4"/>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
-      <c r="G3" s="4"/>
-      <c r="H3" s="4"/>
+      <c r="C3" s="4">
+        <v>0.066</v>
+      </c>
+      <c r="D3" s="4">
+        <v>0.026</v>
+      </c>
+      <c r="E3" s="4">
+        <v>0.005</v>
+      </c>
+      <c r="F3" s="4">
+        <v>0.018</v>
+      </c>
+      <c r="G3" s="4">
+        <v>0.021</v>
+      </c>
+      <c r="H3" s="4">
+        <v>0.001</v>
+      </c>
     </row>
     <row r="4" spans="1:8" s="5" customFormat="1">
       <c r="A4" s="2">
@@ -8785,12 +8797,24 @@
         <f>Table1[[#This Row],[Porcentaje de la muestra '[pct']]]*10000</f>
         <v>500</v>
       </c>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
-      <c r="G4" s="4"/>
-      <c r="H4" s="4"/>
+      <c r="C4" s="4">
+        <v>0.142</v>
+      </c>
+      <c r="D4" s="4">
+        <v>0.167</v>
+      </c>
+      <c r="E4" s="4">
+        <v>0.001</v>
+      </c>
+      <c r="F4" s="4">
+        <v>0.172</v>
+      </c>
+      <c r="G4" s="4">
+        <v>0.215</v>
+      </c>
+      <c r="H4" s="4">
+        <v>0.001</v>
+      </c>
     </row>
     <row r="5" spans="1:8">
       <c r="A5" s="2">
@@ -8800,12 +8824,24 @@
         <f>Table1[[#This Row],[Porcentaje de la muestra '[pct']]]*10000</f>
         <v>1000</v>
       </c>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
-      <c r="G5" s="4"/>
-      <c r="H5" s="4"/>
+      <c r="C5" s="4">
+        <v>0.662</v>
+      </c>
+      <c r="D5" s="4">
+        <v>0.913</v>
+      </c>
+      <c r="E5" s="4">
+        <v>0.001</v>
+      </c>
+      <c r="F5" s="4">
+        <v>1.038</v>
+      </c>
+      <c r="G5" s="4">
+        <v>1.278</v>
+      </c>
+      <c r="H5" s="4">
+        <v>0.001</v>
+      </c>
     </row>
     <row r="6" spans="1:8">
       <c r="A6" s="2">
@@ -8815,12 +8851,24 @@
         <f>Table1[[#This Row],[Porcentaje de la muestra '[pct']]]*10000</f>
         <v>2000</v>
       </c>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4"/>
-      <c r="E6" s="4"/>
-      <c r="F6" s="4"/>
-      <c r="G6" s="4"/>
-      <c r="H6" s="4"/>
+      <c r="C6" s="4">
+        <v>0.895</v>
+      </c>
+      <c r="D6" s="4">
+        <v>1.638</v>
+      </c>
+      <c r="E6" s="4">
+        <v>0.001</v>
+      </c>
+      <c r="F6" s="4">
+        <v>2.066</v>
+      </c>
+      <c r="G6" s="4">
+        <v>1.524</v>
+      </c>
+      <c r="H6" s="4">
+        <v>0.001</v>
+      </c>
     </row>
     <row r="7" spans="1:8">
       <c r="A7" s="2">
@@ -8830,12 +8878,24 @@
         <f>Table1[[#This Row],[Porcentaje de la muestra '[pct']]]*10000</f>
         <v>3000</v>
       </c>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
-      <c r="E7" s="4"/>
-      <c r="F7" s="4"/>
-      <c r="G7" s="4"/>
-      <c r="H7" s="4"/>
+      <c r="C7" s="4">
+        <v>1.210</v>
+      </c>
+      <c r="D7" s="4">
+        <v>1.958</v>
+      </c>
+      <c r="E7" s="4">
+        <v>0.001</v>
+      </c>
+      <c r="F7" s="4">
+        <v>2.970</v>
+      </c>
+      <c r="G7" s="4">
+        <v>2.962</v>
+      </c>
+      <c r="H7" s="4">
+        <v>0.001</v>
+      </c>
     </row>
     <row r="8" spans="1:8">
       <c r="A8" s="2">
@@ -8845,12 +8905,24 @@
         <f>Table1[[#This Row],[Porcentaje de la muestra '[pct']]]*10000</f>
         <v>5000</v>
       </c>
-      <c r="C8" s="4"/>
-      <c r="D8" s="4"/>
-      <c r="E8" s="4"/>
-      <c r="F8" s="4"/>
-      <c r="G8" s="4"/>
-      <c r="H8" s="4"/>
+      <c r="C8" s="4">
+        <v>3.437</v>
+      </c>
+      <c r="D8" s="4">
+        <v>5.939</v>
+      </c>
+      <c r="E8" s="4">
+        <v>0.002</v>
+      </c>
+      <c r="F8" s="4">
+        <v>9.764</v>
+      </c>
+      <c r="G8" s="4">
+        <v>6.541</v>
+      </c>
+      <c r="H8" s="4">
+        <v>0.003</v>
+      </c>
     </row>
     <row r="9" spans="1:8">
       <c r="A9" s="2">
@@ -8860,12 +8932,24 @@
         <f>Table1[[#This Row],[Porcentaje de la muestra '[pct']]]*10000</f>
         <v>8000</v>
       </c>
-      <c r="C9" s="4"/>
-      <c r="D9" s="4"/>
-      <c r="E9" s="4"/>
-      <c r="F9" s="4"/>
-      <c r="G9" s="4"/>
-      <c r="H9" s="4"/>
+      <c r="C9" s="4">
+        <v>5.098</v>
+      </c>
+      <c r="D9" s="4">
+        <v>13.623</v>
+      </c>
+      <c r="E9" s="4">
+        <v>0.004</v>
+      </c>
+      <c r="F9" s="4">
+        <v>28.878</v>
+      </c>
+      <c r="G9" s="4">
+        <v>17.051</v>
+      </c>
+      <c r="H9" s="4">
+        <v>0.003</v>
+      </c>
     </row>
     <row r="10" spans="1:8">
       <c r="A10" s="2">
@@ -8875,12 +8959,24 @@
         <f>Table1[[#This Row],[Porcentaje de la muestra '[pct']]]*10000</f>
         <v>10000</v>
       </c>
-      <c r="C10" s="4"/>
-      <c r="D10" s="4"/>
-      <c r="E10" s="4"/>
-      <c r="F10" s="4"/>
-      <c r="G10" s="4"/>
-      <c r="H10" s="4"/>
+      <c r="C10" s="4">
+        <v>7.550</v>
+      </c>
+      <c r="D10" s="4">
+        <v>20.816</v>
+      </c>
+      <c r="E10" s="4">
+        <v>0.003</v>
+      </c>
+      <c r="F10" s="4">
+        <v>33.326</v>
+      </c>
+      <c r="G10" s="4">
+        <v>12.805</v>
+      </c>
+      <c r="H10" s="4">
+        <v>0.002</v>
+      </c>
     </row>
     <row r="12" spans="1:8" ht="14.25" customHeight="1">
       <c r="C12" s="7" t="s">
@@ -8928,12 +9024,24 @@
         <f>Table13[[#This Row],[Porcentaje de la muestra '[pct']]]*10000</f>
         <v>50</v>
       </c>
-      <c r="C14" s="4"/>
-      <c r="D14" s="4"/>
-      <c r="E14" s="4"/>
-      <c r="F14" s="4"/>
-      <c r="G14" s="4"/>
-      <c r="H14" s="4"/>
+      <c r="C14" s="4">
+        <v>0.026</v>
+      </c>
+      <c r="D14" s="4">
+        <v>0.022</v>
+      </c>
+      <c r="E14" s="4">
+        <v>0.001</v>
+      </c>
+      <c r="F14" s="4">
+        <v>0.019</v>
+      </c>
+      <c r="G14" s="4">
+        <v>0.034</v>
+      </c>
+      <c r="H14" s="4">
+        <v>0.001</v>
+      </c>
     </row>
     <row r="15" spans="1:8" s="5" customFormat="1">
       <c r="A15" s="2">
@@ -8943,12 +9051,24 @@
         <f>Table13[[#This Row],[Porcentaje de la muestra '[pct']]]*10000</f>
         <v>500</v>
       </c>
-      <c r="C15" s="4"/>
-      <c r="D15" s="4"/>
-      <c r="E15" s="4"/>
-      <c r="F15" s="4"/>
-      <c r="G15" s="4"/>
-      <c r="H15" s="4"/>
+      <c r="C15" s="4">
+        <v>0.253</v>
+      </c>
+      <c r="D15" s="4">
+        <v>0.270</v>
+      </c>
+      <c r="E15" s="4">
+        <v>0.001</v>
+      </c>
+      <c r="F15" s="4">
+        <v>0.224</v>
+      </c>
+      <c r="G15" s="4">
+        <v>0.349</v>
+      </c>
+      <c r="H15" s="4">
+        <v>0.001</v>
+      </c>
     </row>
     <row r="16" spans="1:8">
       <c r="A16" s="2">
@@ -8958,12 +9078,24 @@
         <f>Table13[[#This Row],[Porcentaje de la muestra '[pct']]]*10000</f>
         <v>1000</v>
       </c>
-      <c r="C16" s="4"/>
-      <c r="D16" s="4"/>
-      <c r="E16" s="4"/>
-      <c r="F16" s="4"/>
-      <c r="G16" s="4"/>
-      <c r="H16" s="4"/>
+      <c r="C16" s="4">
+        <v>0.478</v>
+      </c>
+      <c r="D16" s="4">
+        <v>0.530</v>
+      </c>
+      <c r="E16" s="4">
+        <v>0.001</v>
+      </c>
+      <c r="F16" s="4">
+        <v>0.435</v>
+      </c>
+      <c r="G16" s="4">
+        <v>0.668</v>
+      </c>
+      <c r="H16" s="4">
+        <v>0.001</v>
+      </c>
     </row>
     <row r="17" spans="1:8">
       <c r="A17" s="2">
@@ -8973,12 +9105,24 @@
         <f>Table13[[#This Row],[Porcentaje de la muestra '[pct']]]*10000</f>
         <v>2000</v>
       </c>
-      <c r="C17" s="4"/>
-      <c r="D17" s="4"/>
-      <c r="E17" s="4"/>
-      <c r="F17" s="4"/>
-      <c r="G17" s="4"/>
-      <c r="H17" s="4"/>
+      <c r="C17" s="4">
+        <v>1.026</v>
+      </c>
+      <c r="D17" s="4">
+        <v>1.619</v>
+      </c>
+      <c r="E17" s="4">
+        <v>0.001</v>
+      </c>
+      <c r="F17" s="4">
+        <v>3.722</v>
+      </c>
+      <c r="G17" s="4">
+        <v>3.109</v>
+      </c>
+      <c r="H17" s="4">
+        <v>0.007</v>
+      </c>
     </row>
     <row r="18" spans="1:8">
       <c r="A18" s="2">
@@ -8988,12 +9132,24 @@
         <f>Table13[[#This Row],[Porcentaje de la muestra '[pct']]]*10000</f>
         <v>3000</v>
       </c>
-      <c r="C18" s="4"/>
-      <c r="D18" s="4"/>
-      <c r="E18" s="4"/>
-      <c r="F18" s="4"/>
-      <c r="G18" s="4"/>
-      <c r="H18" s="4"/>
+      <c r="C18" s="4">
+        <v>2.501</v>
+      </c>
+      <c r="D18" s="4">
+        <v>2.185</v>
+      </c>
+      <c r="E18" s="4">
+        <v>0.006</v>
+      </c>
+      <c r="F18" s="4">
+        <v>2.783</v>
+      </c>
+      <c r="G18" s="4">
+        <v>4.402</v>
+      </c>
+      <c r="H18" s="4">
+        <v>0.002</v>
+      </c>
     </row>
     <row r="19" spans="1:8">
       <c r="A19" s="2">
@@ -9003,12 +9159,24 @@
         <f>Table13[[#This Row],[Porcentaje de la muestra '[pct']]]*10000</f>
         <v>5000</v>
       </c>
-      <c r="C19" s="4"/>
-      <c r="D19" s="4"/>
-      <c r="E19" s="4"/>
-      <c r="F19" s="4"/>
-      <c r="G19" s="4"/>
-      <c r="H19" s="4"/>
+      <c r="C19" s="4">
+        <v>3.856</v>
+      </c>
+      <c r="D19" s="4">
+        <v>3.814</v>
+      </c>
+      <c r="E19" s="4">
+        <v>0.003</v>
+      </c>
+      <c r="F19" s="4">
+        <v>3.639</v>
+      </c>
+      <c r="G19" s="4">
+        <v>4.937</v>
+      </c>
+      <c r="H19" s="4">
+        <v>0.001</v>
+      </c>
     </row>
     <row r="20" spans="1:8">
       <c r="A20" s="2">
@@ -9018,12 +9186,24 @@
         <f>Table13[[#This Row],[Porcentaje de la muestra '[pct']]]*10000</f>
         <v>8000</v>
       </c>
-      <c r="C20" s="4"/>
-      <c r="D20" s="4"/>
-      <c r="E20" s="4"/>
-      <c r="F20" s="4"/>
-      <c r="G20" s="4"/>
-      <c r="H20" s="4"/>
+      <c r="C20" s="4">
+        <v>4.263</v>
+      </c>
+      <c r="D20" s="4">
+        <v>4.310</v>
+      </c>
+      <c r="E20" s="4">
+        <v>0.002</v>
+      </c>
+      <c r="F20" s="4">
+        <v>5.079</v>
+      </c>
+      <c r="G20" s="4">
+        <v>6.075</v>
+      </c>
+      <c r="H20" s="4">
+        <v>0.004</v>
+      </c>
     </row>
     <row r="21" spans="1:8">
       <c r="A21" s="2">
@@ -9033,12 +9213,24 @@
         <f>Table13[[#This Row],[Porcentaje de la muestra '[pct']]]*10000</f>
         <v>10000</v>
       </c>
-      <c r="C21" s="4"/>
-      <c r="D21" s="4"/>
-      <c r="E21" s="4"/>
-      <c r="F21" s="4"/>
-      <c r="G21" s="4"/>
-      <c r="H21" s="4"/>
+      <c r="C21" s="4">
+        <v>5.289</v>
+      </c>
+      <c r="D21" s="4">
+        <v>10.444</v>
+      </c>
+      <c r="E21" s="4">
+        <v>0.002</v>
+      </c>
+      <c r="F21" s="4">
+        <v>99.635</v>
+      </c>
+      <c r="G21" s="4">
+        <v>16.192</v>
+      </c>
+      <c r="H21" s="4">
+        <v>0.005</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -9050,8 +9242,8 @@
   <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="2">
-    <tablePart r:id="rId1"/>
-    <tablePart r:id="rId2"/>
+    <tablePart ns3:id="rId1"/>
+    <tablePart ns3:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>